<commit_message>
update files for ver5.44.0
</commit_message>
<xml_diff>
--- a/sample/ExcelMacro/kabuSTATION_API_function_sample.xlsx
+++ b/sample/ExcelMacro/kabuSTATION_API_function_sample.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\15.MSSOR_Ph2\kabusapi\sample\ExcelMacro\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{816D03C6-A3BF-4FB5-A4EF-E1853DFF697C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F40A181-857F-4251-BF31-8B33B82773EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="787" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="787" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="注文取消" sheetId="1" r:id="rId1"/>
@@ -28,9 +23,10 @@
     <sheet name="優先市場" sheetId="17" r:id="rId13"/>
     <sheet name="ソフトリミット" sheetId="18" r:id="rId14"/>
     <sheet name="プレミアム料取得" sheetId="19" r:id="rId15"/>
-    <sheet name="銘柄登録" sheetId="7" r:id="rId16"/>
-    <sheet name="銘柄登録解除" sheetId="8" r:id="rId17"/>
-    <sheet name="銘柄登録全解除" sheetId="9" r:id="rId18"/>
+    <sheet name="歩み値取得" sheetId="21" r:id="rId16"/>
+    <sheet name="銘柄登録" sheetId="7" r:id="rId17"/>
+    <sheet name="銘柄登録解除" sheetId="8" r:id="rId18"/>
+    <sheet name="銘柄登録全解除" sheetId="9" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">注文約定照会!$B$5:$J$8</definedName>
@@ -56,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1668" uniqueCount="578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1721" uniqueCount="588">
   <si>
     <t>概要</t>
     <rPh sb="0" eb="2">
@@ -3208,6 +3204,79 @@
     <t>東証+</t>
     <rPh sb="0" eb="2">
       <t>トウショウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>歩み値情報を取得する</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>TIMEANDSALES</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>出来時刻</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>出来高</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>出来値</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>※歩み値のリクエストは秒間2件の流量制限を設けております。</t>
+    <rPh sb="1" eb="2">
+      <t>アユ</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>アタイ</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>ビョウカン</t>
+    </rPh>
+    <rPh sb="14" eb="15">
+      <t>ケン</t>
+    </rPh>
+    <rPh sb="16" eb="20">
+      <t>リュウリョウセイゲン</t>
+    </rPh>
+    <rPh sb="21" eb="22">
+      <t>モウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>=TIMEANDSALES(C8,D8)</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>歩み値合計件数</t>
+    <rPh sb="0" eb="1">
+      <t>アユ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>アタイ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ゴウケイ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ケンスウ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>銘柄あたり建玉上限額</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>限週</t>
+    <rPh sb="0" eb="1">
+      <t>カギシュウ</t>
     </rPh>
     <phoneticPr fontId="2"/>
   </si>
@@ -3719,7 +3788,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="189">
+  <cellXfs count="190">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -3918,7 +3987,6 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3993,6 +4061,8 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -4639,22 +4709,22 @@
       <c r="C10" s="65" t="s">
         <v>348</v>
       </c>
-      <c r="D10" s="172" t="s">
+      <c r="D10" s="173" t="s">
         <v>264</v>
       </c>
-      <c r="E10" s="173"/>
+      <c r="E10" s="174"/>
       <c r="H10" s="65" t="s">
         <v>348</v>
       </c>
-      <c r="I10" s="172" t="s">
+      <c r="I10" s="173" t="s">
         <v>264</v>
       </c>
-      <c r="J10" s="173"/>
-      <c r="K10" s="174" t="s">
+      <c r="J10" s="174"/>
+      <c r="K10" s="175" t="s">
         <v>296</v>
       </c>
-      <c r="L10" s="174"/>
-      <c r="M10" s="174"/>
+      <c r="L10" s="175"/>
+      <c r="M10" s="175"/>
     </row>
     <row r="11" spans="2:14">
       <c r="B11" s="80" t="s">
@@ -4670,18 +4740,18 @@
       <c r="G11" s="86" t="s">
         <v>312</v>
       </c>
-      <c r="H11" s="142" t="s">
+      <c r="H11" s="141" t="s">
         <v>310</v>
       </c>
       <c r="I11" s="82" t="s">
         <v>364</v>
       </c>
       <c r="J11" s="74"/>
-      <c r="K11" s="175" t="s">
+      <c r="K11" s="176" t="s">
         <v>544</v>
       </c>
-      <c r="L11" s="176"/>
-      <c r="M11" s="177"/>
+      <c r="L11" s="177"/>
+      <c r="M11" s="178"/>
     </row>
     <row r="12" spans="2:14">
       <c r="B12" s="83"/>
@@ -4693,16 +4763,16 @@
       </c>
       <c r="E12" s="74"/>
       <c r="G12" s="84"/>
-      <c r="H12" s="142" t="s">
+      <c r="H12" s="141" t="s">
         <v>365</v>
       </c>
       <c r="I12" s="82" t="s">
         <v>366</v>
       </c>
       <c r="J12" s="74"/>
-      <c r="K12" s="178"/>
-      <c r="L12" s="179"/>
-      <c r="M12" s="180"/>
+      <c r="K12" s="179"/>
+      <c r="L12" s="180"/>
+      <c r="M12" s="181"/>
     </row>
     <row r="13" spans="2:14">
       <c r="B13" s="83"/>
@@ -4714,17 +4784,17 @@
       </c>
       <c r="E13" s="74"/>
       <c r="G13" s="84"/>
-      <c r="H13" s="143" t="s">
+      <c r="H13" s="142" t="s">
         <v>538</v>
       </c>
-      <c r="I13" s="144" t="s">
+      <c r="I13" s="143" t="s">
         <v>541</v>
       </c>
       <c r="J13" s="74"/>
-      <c r="K13" s="178"/>
-      <c r="L13" s="179"/>
-      <c r="M13" s="180"/>
-      <c r="N13" s="141"/>
+      <c r="K13" s="179"/>
+      <c r="L13" s="180"/>
+      <c r="M13" s="181"/>
+      <c r="N13" s="140"/>
     </row>
     <row r="14" spans="2:14">
       <c r="B14" s="83"/>
@@ -4736,17 +4806,17 @@
       </c>
       <c r="E14" s="74"/>
       <c r="G14" s="84"/>
-      <c r="H14" s="143" t="s">
+      <c r="H14" s="142" t="s">
         <v>539</v>
       </c>
-      <c r="I14" s="144" t="s">
+      <c r="I14" s="143" t="s">
         <v>542</v>
       </c>
       <c r="J14" s="74"/>
-      <c r="K14" s="178"/>
-      <c r="L14" s="179"/>
-      <c r="M14" s="180"/>
-      <c r="N14" s="141"/>
+      <c r="K14" s="179"/>
+      <c r="L14" s="180"/>
+      <c r="M14" s="181"/>
+      <c r="N14" s="140"/>
     </row>
     <row r="15" spans="2:14">
       <c r="B15" s="83"/>
@@ -4758,17 +4828,17 @@
       </c>
       <c r="E15" s="74"/>
       <c r="G15" s="84"/>
-      <c r="H15" s="143" t="s">
+      <c r="H15" s="142" t="s">
         <v>540</v>
       </c>
-      <c r="I15" s="144" t="s">
+      <c r="I15" s="143" t="s">
         <v>543</v>
       </c>
       <c r="J15" s="74"/>
-      <c r="K15" s="178"/>
-      <c r="L15" s="179"/>
-      <c r="M15" s="180"/>
-      <c r="N15" s="141"/>
+      <c r="K15" s="179"/>
+      <c r="L15" s="180"/>
+      <c r="M15" s="181"/>
+      <c r="N15" s="140"/>
     </row>
     <row r="16" spans="2:14">
       <c r="B16" s="83"/>
@@ -4780,16 +4850,16 @@
       </c>
       <c r="E16" s="74"/>
       <c r="G16" s="84"/>
-      <c r="H16" s="142" t="s">
+      <c r="H16" s="141" t="s">
         <v>367</v>
       </c>
       <c r="I16" s="82" t="s">
         <v>368</v>
       </c>
       <c r="J16" s="74"/>
-      <c r="K16" s="178"/>
-      <c r="L16" s="179"/>
-      <c r="M16" s="180"/>
+      <c r="K16" s="179"/>
+      <c r="L16" s="180"/>
+      <c r="M16" s="181"/>
     </row>
     <row r="17" spans="2:18">
       <c r="B17" s="83"/>
@@ -4801,16 +4871,16 @@
       </c>
       <c r="E17" s="74"/>
       <c r="G17" s="84"/>
-      <c r="H17" s="142" t="s">
+      <c r="H17" s="141" t="s">
         <v>369</v>
       </c>
       <c r="I17" s="82" t="s">
         <v>194</v>
       </c>
       <c r="J17" s="74"/>
-      <c r="K17" s="178"/>
-      <c r="L17" s="179"/>
-      <c r="M17" s="180"/>
+      <c r="K17" s="179"/>
+      <c r="L17" s="180"/>
+      <c r="M17" s="181"/>
     </row>
     <row r="18" spans="2:18">
       <c r="B18" s="83"/>
@@ -4822,16 +4892,16 @@
       </c>
       <c r="E18" s="74"/>
       <c r="G18" s="85"/>
-      <c r="H18" s="142" t="s">
+      <c r="H18" s="141" t="s">
         <v>370</v>
       </c>
       <c r="I18" s="82" t="s">
         <v>371</v>
       </c>
       <c r="J18" s="74"/>
-      <c r="K18" s="181"/>
-      <c r="L18" s="182"/>
-      <c r="M18" s="183"/>
+      <c r="K18" s="182"/>
+      <c r="L18" s="183"/>
+      <c r="M18" s="184"/>
     </row>
     <row r="19" spans="2:18">
       <c r="B19" s="84"/>
@@ -7377,7 +7447,7 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:16">
-      <c r="B2" s="114" t="s">
+      <c r="B2" s="146" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="114" t="s">
@@ -7388,7 +7458,7 @@
       <c r="F2" s="116"/>
     </row>
     <row r="3" spans="2:16">
-      <c r="B3" s="118" t="s">
+      <c r="B3" s="147" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="114" t="s">
@@ -7404,17 +7474,17 @@
       </c>
     </row>
     <row r="6" spans="2:16">
-      <c r="C6" s="119" t="s">
+      <c r="C6" s="118" t="s">
         <v>509</v>
       </c>
     </row>
     <row r="7" spans="2:16">
-      <c r="C7" s="120" t="s">
+      <c r="C7" s="119" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="8" spans="2:16">
-      <c r="C8" s="121" t="s">
+      <c r="C8" s="120" t="s">
         <v>291</v>
       </c>
     </row>
@@ -7429,64 +7499,64 @@
       <c r="C12" s="99" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="122" t="s">
+      <c r="D12" s="121" t="s">
         <v>520</v>
       </c>
     </row>
     <row r="13" spans="2:16">
-      <c r="D13" s="123"/>
-      <c r="E13" s="124"/>
-      <c r="F13" s="125"/>
-      <c r="G13" s="126" t="s">
+      <c r="D13" s="122"/>
+      <c r="E13" s="123"/>
+      <c r="F13" s="124"/>
+      <c r="G13" s="125" t="s">
         <v>521</v>
       </c>
-      <c r="H13" s="125"/>
-      <c r="I13" s="127"/>
-      <c r="J13" s="125"/>
-      <c r="K13" s="125"/>
-      <c r="L13" s="125"/>
-      <c r="M13" s="126" t="s">
+      <c r="H13" s="124"/>
+      <c r="I13" s="126"/>
+      <c r="J13" s="124"/>
+      <c r="K13" s="124"/>
+      <c r="L13" s="124"/>
+      <c r="M13" s="125" t="s">
         <v>522</v>
       </c>
-      <c r="N13" s="127"/>
-      <c r="O13" s="123"/>
-      <c r="P13" s="123"/>
+      <c r="N13" s="126"/>
+      <c r="O13" s="122"/>
+      <c r="P13" s="122"/>
     </row>
     <row r="14" spans="2:16">
-      <c r="C14" s="119" t="s">
+      <c r="C14" s="118" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="128" t="s">
+      <c r="D14" s="127" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="137" t="s">
+      <c r="E14" s="136" t="s">
         <v>510</v>
       </c>
-      <c r="F14" s="137" t="s">
+      <c r="F14" s="136" t="s">
         <v>514</v>
       </c>
-      <c r="G14" s="137" t="s">
+      <c r="G14" s="136" t="s">
         <v>516</v>
       </c>
-      <c r="H14" s="137" t="s">
+      <c r="H14" s="136" t="s">
         <v>517</v>
       </c>
-      <c r="I14" s="137" t="s">
+      <c r="I14" s="136" t="s">
         <v>528</v>
       </c>
-      <c r="J14" s="137" t="s">
+      <c r="J14" s="136" t="s">
         <v>510</v>
       </c>
-      <c r="K14" s="137" t="s">
+      <c r="K14" s="136" t="s">
         <v>514</v>
       </c>
-      <c r="L14" s="137" t="s">
+      <c r="L14" s="136" t="s">
         <v>516</v>
       </c>
-      <c r="M14" s="137" t="s">
+      <c r="M14" s="136" t="s">
         <v>517</v>
       </c>
-      <c r="N14" s="137" t="s">
+      <c r="N14" s="136" t="s">
         <v>528</v>
       </c>
     </row>
@@ -7495,159 +7565,159 @@
         <f>"(D"&amp;ROW()&amp;"に関数入力)"</f>
         <v>(D15に関数入力)</v>
       </c>
-      <c r="D15" s="129" t="s">
+      <c r="D15" s="128" t="s">
         <v>519</v>
       </c>
-      <c r="E15" s="129" t="s">
+      <c r="E15" s="128" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="129" t="s">
+      <c r="F15" s="128" t="s">
         <v>12</v>
       </c>
-      <c r="G15" s="129" t="s">
+      <c r="G15" s="128" t="s">
         <v>12</v>
       </c>
-      <c r="H15" s="129" t="s">
+      <c r="H15" s="128" t="s">
         <v>12</v>
       </c>
-      <c r="I15" s="129" t="s">
+      <c r="I15" s="128" t="s">
         <v>12</v>
       </c>
-      <c r="J15" s="129" t="s">
+      <c r="J15" s="128" t="s">
         <v>12</v>
       </c>
-      <c r="K15" s="129" t="s">
+      <c r="K15" s="128" t="s">
         <v>12</v>
       </c>
-      <c r="L15" s="129" t="s">
+      <c r="L15" s="128" t="s">
         <v>12</v>
       </c>
-      <c r="M15" s="129" t="s">
+      <c r="M15" s="128" t="s">
         <v>12</v>
       </c>
-      <c r="N15" s="129" t="s">
+      <c r="N15" s="128" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="2:16">
-      <c r="D16" s="129"/>
-      <c r="E16" s="129"/>
-      <c r="F16" s="129"/>
-      <c r="G16" s="129"/>
-      <c r="H16" s="129"/>
-      <c r="I16" s="129"/>
-      <c r="J16" s="129"/>
-      <c r="K16" s="129"/>
-      <c r="L16" s="129"/>
-      <c r="M16" s="129"/>
-      <c r="N16" s="129"/>
+      <c r="D16" s="128"/>
+      <c r="E16" s="128"/>
+      <c r="F16" s="128"/>
+      <c r="G16" s="128"/>
+      <c r="H16" s="128"/>
+      <c r="I16" s="128"/>
+      <c r="J16" s="128"/>
+      <c r="K16" s="128"/>
+      <c r="L16" s="128"/>
+      <c r="M16" s="128"/>
+      <c r="N16" s="128"/>
     </row>
     <row r="17" spans="3:14">
-      <c r="D17" s="129"/>
-      <c r="E17" s="129"/>
-      <c r="F17" s="129"/>
-      <c r="G17" s="129"/>
-      <c r="H17" s="129"/>
-      <c r="I17" s="129"/>
-      <c r="J17" s="129"/>
-      <c r="K17" s="129"/>
-      <c r="L17" s="129"/>
-      <c r="M17" s="129"/>
-      <c r="N17" s="129"/>
+      <c r="D17" s="128"/>
+      <c r="E17" s="128"/>
+      <c r="F17" s="128"/>
+      <c r="G17" s="128"/>
+      <c r="H17" s="128"/>
+      <c r="I17" s="128"/>
+      <c r="J17" s="128"/>
+      <c r="K17" s="128"/>
+      <c r="L17" s="128"/>
+      <c r="M17" s="128"/>
+      <c r="N17" s="128"/>
     </row>
     <row r="18" spans="3:14">
-      <c r="D18" s="129"/>
-      <c r="E18" s="129"/>
-      <c r="F18" s="129"/>
-      <c r="G18" s="129"/>
-      <c r="H18" s="129"/>
-      <c r="I18" s="129"/>
-      <c r="J18" s="129"/>
-      <c r="K18" s="129"/>
-      <c r="L18" s="129"/>
-      <c r="M18" s="129"/>
-      <c r="N18" s="129"/>
+      <c r="D18" s="128"/>
+      <c r="E18" s="128"/>
+      <c r="F18" s="128"/>
+      <c r="G18" s="128"/>
+      <c r="H18" s="128"/>
+      <c r="I18" s="128"/>
+      <c r="J18" s="128"/>
+      <c r="K18" s="128"/>
+      <c r="L18" s="128"/>
+      <c r="M18" s="128"/>
+      <c r="N18" s="128"/>
     </row>
     <row r="19" spans="3:14">
-      <c r="D19" s="129"/>
-      <c r="E19" s="129"/>
-      <c r="F19" s="129"/>
-      <c r="G19" s="129"/>
-      <c r="H19" s="129"/>
-      <c r="I19" s="129"/>
-      <c r="J19" s="129"/>
-      <c r="K19" s="129"/>
-      <c r="L19" s="129"/>
-      <c r="M19" s="129"/>
-      <c r="N19" s="129"/>
+      <c r="D19" s="128"/>
+      <c r="E19" s="128"/>
+      <c r="F19" s="128"/>
+      <c r="G19" s="128"/>
+      <c r="H19" s="128"/>
+      <c r="I19" s="128"/>
+      <c r="J19" s="128"/>
+      <c r="K19" s="128"/>
+      <c r="L19" s="128"/>
+      <c r="M19" s="128"/>
+      <c r="N19" s="128"/>
     </row>
     <row r="20" spans="3:14">
-      <c r="D20" s="129"/>
-      <c r="E20" s="129"/>
-      <c r="F20" s="129"/>
-      <c r="G20" s="129"/>
-      <c r="H20" s="129"/>
-      <c r="I20" s="129"/>
-      <c r="J20" s="129"/>
-      <c r="K20" s="129"/>
-      <c r="L20" s="129"/>
-      <c r="M20" s="129"/>
-      <c r="N20" s="129"/>
+      <c r="D20" s="128"/>
+      <c r="E20" s="128"/>
+      <c r="F20" s="128"/>
+      <c r="G20" s="128"/>
+      <c r="H20" s="128"/>
+      <c r="I20" s="128"/>
+      <c r="J20" s="128"/>
+      <c r="K20" s="128"/>
+      <c r="L20" s="128"/>
+      <c r="M20" s="128"/>
+      <c r="N20" s="128"/>
     </row>
     <row r="23" spans="3:14">
-      <c r="C23" s="130" t="s">
+      <c r="C23" s="129" t="s">
         <v>510</v>
       </c>
-      <c r="D23" s="131" t="s">
+      <c r="D23" s="130" t="s">
         <v>511</v>
       </c>
-      <c r="E23" s="184" t="s">
+      <c r="E23" s="185" t="s">
         <v>512</v>
       </c>
-      <c r="F23" s="185"/>
+      <c r="F23" s="186"/>
     </row>
     <row r="24" spans="3:14">
-      <c r="C24" s="140"/>
-      <c r="D24" s="133" t="s">
+      <c r="C24" s="139"/>
+      <c r="D24" s="132" t="s">
         <v>533</v>
       </c>
-      <c r="E24" s="186" t="s">
+      <c r="E24" s="187" t="s">
         <v>534</v>
       </c>
-      <c r="F24" s="186"/>
+      <c r="F24" s="187"/>
     </row>
     <row r="25" spans="3:14">
-      <c r="C25" s="132"/>
-      <c r="D25" s="133">
+      <c r="C25" s="131"/>
+      <c r="D25" s="132">
         <v>0</v>
       </c>
-      <c r="E25" s="187" t="s">
+      <c r="E25" s="188" t="s">
         <v>535</v>
       </c>
-      <c r="F25" s="187"/>
+      <c r="F25" s="188"/>
     </row>
     <row r="26" spans="3:14">
-      <c r="C26" s="132"/>
-      <c r="D26" s="134">
+      <c r="C26" s="131"/>
+      <c r="D26" s="133">
         <v>1</v>
       </c>
-      <c r="E26" s="188" t="s">
+      <c r="E26" s="189" t="s">
         <v>536</v>
       </c>
-      <c r="F26" s="188"/>
+      <c r="F26" s="189"/>
     </row>
     <row r="27" spans="3:14">
-      <c r="C27" s="135"/>
-      <c r="D27" s="133">
+      <c r="C27" s="134"/>
+      <c r="D27" s="132">
         <v>2</v>
       </c>
-      <c r="E27" s="187" t="s">
+      <c r="E27" s="188" t="s">
         <v>537</v>
       </c>
-      <c r="F27" s="187"/>
+      <c r="F27" s="188"/>
     </row>
     <row r="29" spans="3:14">
-      <c r="D29" s="138" t="s">
+      <c r="D29" s="137" t="s">
         <v>527</v>
       </c>
       <c r="E29" s="117" t="s">
@@ -7655,7 +7725,7 @@
       </c>
     </row>
     <row r="30" spans="3:14">
-      <c r="D30" s="139"/>
+      <c r="D30" s="138"/>
       <c r="E30" s="117" t="s">
         <v>524</v>
       </c>
@@ -7671,7 +7741,7 @@
       </c>
     </row>
     <row r="33" spans="4:5">
-      <c r="D33" s="139" t="s">
+      <c r="D33" s="138" t="s">
         <v>532</v>
       </c>
       <c r="E33" s="117" t="s">
@@ -7679,7 +7749,7 @@
       </c>
     </row>
     <row r="34" spans="4:5">
-      <c r="D34" s="139" t="s">
+      <c r="D34" s="138" t="s">
         <v>530</v>
       </c>
       <c r="E34" s="117" t="s">
@@ -7687,7 +7757,7 @@
       </c>
     </row>
     <row r="40" spans="4:5">
-      <c r="D40" s="136"/>
+      <c r="D40" s="135"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -7704,6 +7774,279 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E9CBCEE-3B31-4688-94AB-19F8F6D98371}">
+  <dimension ref="A1:I33"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="3" max="5" width="17.125" customWidth="1"/>
+    <col min="6" max="6" width="18.375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="117"/>
+      <c r="B1" s="117"/>
+      <c r="C1" s="117"/>
+      <c r="D1" s="117"/>
+      <c r="E1" s="117"/>
+      <c r="F1" s="117"/>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="117"/>
+      <c r="B2" s="146" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="114" t="s">
+        <v>578</v>
+      </c>
+      <c r="D2" s="115"/>
+      <c r="E2" s="115"/>
+      <c r="F2" s="116"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="117"/>
+      <c r="B3" s="147" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="114" t="s">
+        <v>579</v>
+      </c>
+      <c r="D3" s="115"/>
+      <c r="E3" s="115"/>
+      <c r="F3" s="116"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="B5" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="B6" s="6"/>
+      <c r="C6" s="6" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="B7" s="6"/>
+      <c r="C7" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="B8" s="6"/>
+      <c r="C8" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="D8" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="C10" s="31" t="s">
+        <v>198</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>191</v>
+      </c>
+      <c r="E10" s="31" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="C11" s="32" t="s">
+        <v>260</v>
+      </c>
+      <c r="D11" s="23">
+        <v>1</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="C12" s="33" t="s">
+        <v>261</v>
+      </c>
+      <c r="D12" s="23">
+        <v>3</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="C13" s="33"/>
+      <c r="D13" s="23">
+        <v>5</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="C14" s="34"/>
+      <c r="D14" s="23">
+        <v>6</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="C15" s="35" t="s">
+        <v>262</v>
+      </c>
+      <c r="D15" s="23">
+        <v>2</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="C16" s="33" t="s">
+        <v>263</v>
+      </c>
+      <c r="D16" s="23">
+        <v>23</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9">
+      <c r="C17" s="34"/>
+      <c r="D17" s="23">
+        <v>24</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9">
+      <c r="B19" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9">
+      <c r="C21" t="s">
+        <v>196</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9">
+      <c r="C22" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9">
+      <c r="C23" s="27" t="str">
+        <f>"(D"&amp;ROW()&amp;"に関数入力)"</f>
+        <v>(D23に関数入力)</v>
+      </c>
+      <c r="D23" s="7">
+        <v>8306</v>
+      </c>
+      <c r="E23" s="23">
+        <v>1</v>
+      </c>
+      <c r="F23" s="23">
+        <v>5</v>
+      </c>
+      <c r="G23" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="H23" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="I23" s="23" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9">
+      <c r="G24" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="H24" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="I24" s="23" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9">
+      <c r="G25" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="H25" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="I25" s="23" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9">
+      <c r="G26" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="H26" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="I26" s="23" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9">
+      <c r="G27" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="H27" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="I27" s="23" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33" t="s">
+        <v>583</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{6A91A987-CD97-45A9-807C-CA71CE2664E6}">
+      <formula1>"1,3,5,6,2,23,24"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A2:H40"/>
@@ -8068,10 +8411,11 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <sheetPr codeName="Sheet12"/>
   <dimension ref="A2:H40"/>
@@ -8397,10 +8741,11 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <sheetPr codeName="Sheet13"/>
   <dimension ref="A2:H20"/>
@@ -8712,12 +9057,12 @@
       </c>
     </row>
     <row r="20" spans="1:8">
-      <c r="H20" s="145" t="s">
+      <c r="H20" s="144" t="s">
         <v>549</v>
       </c>
     </row>
     <row r="21" spans="1:8">
-      <c r="H21" s="145" t="s">
+      <c r="H21" s="144" t="s">
         <v>550</v>
       </c>
     </row>
@@ -8736,7 +9081,7 @@
       <c r="D23" s="31" t="s">
         <v>264</v>
       </c>
-      <c r="H23" s="146" t="s">
+      <c r="H23" s="145" t="s">
         <v>551</v>
       </c>
     </row>
@@ -10653,12 +10998,13 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A2:AA28"/>
+  <dimension ref="A2:AC28"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="13.375" customWidth="1"/>
@@ -10674,13 +11020,15 @@
     <col min="12" max="13" width="8.375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.25" bestFit="1" customWidth="1"/>
     <col min="15" max="18" width="18.25" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.25" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.25" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.25" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="17.25" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="6.75" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="21.375" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="8.375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.25" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.25" customWidth="1"/>
+    <col min="25" max="26" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.25" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="6.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8">
@@ -10834,7 +11182,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="17" spans="1:27">
+    <row r="17" spans="1:29">
       <c r="C17" s="34"/>
       <c r="D17" s="23">
         <v>24</v>
@@ -10843,15 +11191,15 @@
         <v>259</v>
       </c>
     </row>
-    <row r="19" spans="1:27">
+    <row r="19" spans="1:29">
       <c r="B19" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:27">
+    <row r="20" spans="1:29">
       <c r="B20" s="5"/>
     </row>
-    <row r="21" spans="1:27">
+    <row r="21" spans="1:29">
       <c r="B21" s="5"/>
       <c r="C21" t="s">
         <v>196</v>
@@ -10860,7 +11208,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="22" spans="1:27">
+    <row r="22" spans="1:29">
       <c r="C22" s="6" t="s">
         <v>10</v>
       </c>
@@ -10910,34 +11258,40 @@
         <v>97</v>
       </c>
       <c r="S22" s="8" t="s">
+        <v>586</v>
+      </c>
+      <c r="T22" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="T22" s="8" t="s">
+      <c r="U22" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="U22" s="8" t="s">
+      <c r="V22" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="V22" s="8" t="s">
+      <c r="W22" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="W22" s="8" t="s">
+      <c r="X22" s="8" t="s">
+        <v>587</v>
+      </c>
+      <c r="Y22" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="X22" s="8" t="s">
+      <c r="Z22" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="Y22" s="8" t="s">
+      <c r="AA22" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="Z22" s="8" t="s">
+      <c r="AB22" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="AA22" s="8" t="s">
+      <c r="AC22" s="8" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="23" spans="1:27">
+    <row r="23" spans="1:29">
       <c r="A23" s="6"/>
       <c r="C23" s="27" t="str">
         <f>"(D"&amp;ROW()&amp;"に関数入力)"</f>
@@ -11015,8 +11369,14 @@
       <c r="AA23" s="7" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="24" spans="1:27">
+      <c r="AB23" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="AC23" s="7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24" spans="1:29">
       <c r="A24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
@@ -11042,23 +11402,25 @@
       <c r="Y24" s="6"/>
       <c r="Z24" s="6"/>
       <c r="AA24" s="6"/>
-    </row>
-    <row r="25" spans="1:27">
+      <c r="AB24" s="6"/>
+      <c r="AC24" s="6"/>
+    </row>
+    <row r="25" spans="1:29">
       <c r="B25" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="26" spans="1:27">
+    <row r="26" spans="1:29">
       <c r="B26" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="27" spans="1:27">
+    <row r="27" spans="1:29">
       <c r="B27" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="28" spans="1:27">
+    <row r="28" spans="1:29">
       <c r="B28" s="89" t="s">
         <v>307</v>
       </c>
@@ -11074,6 +11436,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -11229,89 +11592,89 @@
       <c r="C11" s="65" t="s">
         <v>301</v>
       </c>
-      <c r="D11" s="155" t="s">
+      <c r="D11" s="156" t="s">
         <v>295</v>
       </c>
-      <c r="E11" s="156"/>
-      <c r="F11" s="155" t="s">
+      <c r="E11" s="157"/>
+      <c r="F11" s="156" t="s">
         <v>296</v>
       </c>
-      <c r="G11" s="156"/>
+      <c r="G11" s="157"/>
       <c r="L11" t="s">
         <v>504</v>
       </c>
     </row>
     <row r="12" spans="2:12">
-      <c r="B12" s="171" t="s">
+      <c r="B12" s="172" t="s">
         <v>275</v>
       </c>
       <c r="C12" s="42">
         <v>0</v>
       </c>
-      <c r="D12" s="167" t="s">
+      <c r="D12" s="168" t="s">
         <v>201</v>
       </c>
-      <c r="E12" s="168"/>
-      <c r="F12" s="157" t="s">
+      <c r="E12" s="169"/>
+      <c r="F12" s="158" t="s">
         <v>297</v>
       </c>
-      <c r="G12" s="158"/>
+      <c r="G12" s="159"/>
       <c r="L12" t="s">
         <v>505</v>
       </c>
     </row>
     <row r="13" spans="2:12">
-      <c r="B13" s="171"/>
+      <c r="B13" s="172"/>
       <c r="C13" s="42">
         <v>1</v>
       </c>
-      <c r="D13" s="167" t="s">
+      <c r="D13" s="168" t="s">
         <v>200</v>
       </c>
-      <c r="E13" s="168"/>
-      <c r="F13" s="159" t="s">
+      <c r="E13" s="169"/>
+      <c r="F13" s="160" t="s">
         <v>304</v>
       </c>
-      <c r="G13" s="160"/>
+      <c r="G13" s="161"/>
       <c r="L13" t="s">
         <v>506</v>
       </c>
     </row>
     <row r="14" spans="2:12">
-      <c r="B14" s="171"/>
+      <c r="B14" s="172"/>
       <c r="C14" s="42">
         <v>2</v>
       </c>
-      <c r="D14" s="167" t="s">
+      <c r="D14" s="168" t="s">
         <v>199</v>
       </c>
-      <c r="E14" s="168"/>
-      <c r="F14" s="159"/>
-      <c r="G14" s="160"/>
+      <c r="E14" s="169"/>
+      <c r="F14" s="160"/>
+      <c r="G14" s="161"/>
     </row>
     <row r="15" spans="2:12">
-      <c r="B15" s="171"/>
+      <c r="B15" s="172"/>
       <c r="C15" s="42">
         <v>3</v>
       </c>
-      <c r="D15" s="167" t="s">
+      <c r="D15" s="168" t="s">
         <v>262</v>
       </c>
-      <c r="E15" s="168"/>
-      <c r="F15" s="159"/>
-      <c r="G15" s="160"/>
+      <c r="E15" s="169"/>
+      <c r="F15" s="160"/>
+      <c r="G15" s="161"/>
     </row>
     <row r="16" spans="2:12">
-      <c r="B16" s="171"/>
+      <c r="B16" s="172"/>
       <c r="C16" s="42">
         <v>4</v>
       </c>
-      <c r="D16" s="167" t="s">
+      <c r="D16" s="168" t="s">
         <v>263</v>
       </c>
-      <c r="E16" s="168"/>
-      <c r="F16" s="161"/>
-      <c r="G16" s="162"/>
+      <c r="E16" s="169"/>
+      <c r="F16" s="162"/>
+      <c r="G16" s="163"/>
     </row>
     <row r="17" spans="2:7">
       <c r="B17" s="58" t="s">
@@ -11366,30 +11729,30 @@
       <c r="G20" s="62"/>
     </row>
     <row r="21" spans="2:7">
-      <c r="B21" s="169" t="s">
+      <c r="B21" s="170" t="s">
         <v>284</v>
       </c>
       <c r="C21" s="42" t="b">
         <v>1</v>
       </c>
-      <c r="D21" s="167" t="s">
+      <c r="D21" s="168" t="s">
         <v>302</v>
       </c>
-      <c r="E21" s="168"/>
+      <c r="E21" s="169"/>
       <c r="F21" s="66" t="s">
         <v>297</v>
       </c>
       <c r="G21" s="67"/>
     </row>
     <row r="22" spans="2:7">
-      <c r="B22" s="169"/>
+      <c r="B22" s="170"/>
       <c r="C22" s="42" t="b">
         <v>0</v>
       </c>
-      <c r="D22" s="167" t="s">
+      <c r="D22" s="168" t="s">
         <v>303</v>
       </c>
-      <c r="E22" s="168"/>
+      <c r="E22" s="169"/>
       <c r="F22" s="68" t="s">
         <v>305</v>
       </c>
@@ -11412,130 +11775,130 @@
       <c r="G23" s="64"/>
     </row>
     <row r="24" spans="2:7">
-      <c r="B24" s="169" t="s">
+      <c r="B24" s="170" t="s">
         <v>287</v>
       </c>
       <c r="C24" s="41">
         <v>1</v>
       </c>
-      <c r="D24" s="165" t="s">
+      <c r="D24" s="166" t="s">
         <v>285</v>
       </c>
-      <c r="E24" s="166"/>
-      <c r="F24" s="163" t="s">
+      <c r="E24" s="167"/>
+      <c r="F24" s="164" t="s">
         <v>297</v>
       </c>
-      <c r="G24" s="164"/>
+      <c r="G24" s="165"/>
     </row>
     <row r="25" spans="2:7">
-      <c r="B25" s="169"/>
+      <c r="B25" s="170"/>
       <c r="C25" s="41">
         <v>2</v>
       </c>
-      <c r="D25" s="153" t="s">
+      <c r="D25" s="154" t="s">
         <v>276</v>
       </c>
-      <c r="E25" s="154"/>
-      <c r="F25" s="147" t="s">
+      <c r="E25" s="155"/>
+      <c r="F25" s="148" t="s">
         <v>304</v>
       </c>
-      <c r="G25" s="148"/>
+      <c r="G25" s="149"/>
     </row>
     <row r="26" spans="2:7">
-      <c r="B26" s="169"/>
+      <c r="B26" s="170"/>
       <c r="C26" s="41">
         <v>3</v>
       </c>
-      <c r="D26" s="153" t="s">
+      <c r="D26" s="154" t="s">
         <v>277</v>
       </c>
-      <c r="E26" s="154"/>
-      <c r="F26" s="147"/>
-      <c r="G26" s="148"/>
+      <c r="E26" s="155"/>
+      <c r="F26" s="148"/>
+      <c r="G26" s="149"/>
     </row>
     <row r="27" spans="2:7">
-      <c r="B27" s="169"/>
+      <c r="B27" s="170"/>
       <c r="C27" s="41">
         <v>4</v>
       </c>
-      <c r="D27" s="153" t="s">
+      <c r="D27" s="154" t="s">
         <v>278</v>
       </c>
-      <c r="E27" s="154"/>
-      <c r="F27" s="147"/>
-      <c r="G27" s="148"/>
+      <c r="E27" s="155"/>
+      <c r="F27" s="148"/>
+      <c r="G27" s="149"/>
     </row>
     <row r="28" spans="2:7">
-      <c r="B28" s="169"/>
+      <c r="B28" s="170"/>
       <c r="C28" s="41">
         <v>5</v>
       </c>
-      <c r="D28" s="153" t="s">
+      <c r="D28" s="154" t="s">
         <v>279</v>
       </c>
-      <c r="E28" s="154"/>
-      <c r="F28" s="151"/>
-      <c r="G28" s="152"/>
+      <c r="E28" s="155"/>
+      <c r="F28" s="152"/>
+      <c r="G28" s="153"/>
     </row>
     <row r="29" spans="2:7">
-      <c r="B29" s="169" t="s">
+      <c r="B29" s="170" t="s">
         <v>288</v>
       </c>
       <c r="C29" s="41">
         <v>1</v>
       </c>
-      <c r="D29" s="165" t="s">
+      <c r="D29" s="166" t="s">
         <v>286</v>
       </c>
-      <c r="E29" s="166"/>
-      <c r="F29" s="163" t="s">
+      <c r="E29" s="167"/>
+      <c r="F29" s="164" t="s">
         <v>297</v>
       </c>
-      <c r="G29" s="164"/>
+      <c r="G29" s="165"/>
     </row>
     <row r="30" spans="2:7">
-      <c r="B30" s="169"/>
+      <c r="B30" s="170"/>
       <c r="C30" s="41">
         <v>2</v>
       </c>
-      <c r="D30" s="153" t="s">
+      <c r="D30" s="154" t="s">
         <v>280</v>
       </c>
-      <c r="E30" s="154"/>
-      <c r="F30" s="147" t="s">
+      <c r="E30" s="155"/>
+      <c r="F30" s="148" t="s">
         <v>304</v>
       </c>
-      <c r="G30" s="148"/>
+      <c r="G30" s="149"/>
     </row>
     <row r="31" spans="2:7">
-      <c r="B31" s="170" t="s">
+      <c r="B31" s="171" t="s">
         <v>289</v>
       </c>
       <c r="C31" s="41">
         <v>2</v>
       </c>
-      <c r="D31" s="153" t="s">
+      <c r="D31" s="154" t="s">
         <v>281</v>
       </c>
-      <c r="E31" s="154"/>
-      <c r="F31" s="149" t="s">
+      <c r="E31" s="155"/>
+      <c r="F31" s="150" t="s">
         <v>297</v>
       </c>
-      <c r="G31" s="150"/>
+      <c r="G31" s="151"/>
     </row>
     <row r="32" spans="2:7">
-      <c r="B32" s="170"/>
+      <c r="B32" s="171"/>
       <c r="C32" s="41">
         <v>3</v>
       </c>
-      <c r="D32" s="153" t="s">
+      <c r="D32" s="154" t="s">
         <v>282</v>
       </c>
-      <c r="E32" s="154"/>
-      <c r="F32" s="151" t="s">
+      <c r="E32" s="155"/>
+      <c r="F32" s="152" t="s">
         <v>304</v>
       </c>
-      <c r="G32" s="152"/>
+      <c r="G32" s="153"/>
     </row>
     <row r="33" spans="1:37">
       <c r="B33" s="6"/>
@@ -22984,6 +23347,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -23203,6 +23567,7 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -23386,6 +23751,7 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -23545,5 +23911,6 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>